<commit_message>
modificando la plantilla de nomina
</commit_message>
<xml_diff>
--- a/RN_GC/web/resources/Archivos/Plantilla_Nomina.xlsx
+++ b/RN_GC/web/resources/Archivos/Plantilla_Nomina.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Documents\NetBeansProjects\RN_GC\web\resources\Archivos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698407EF-6F1D-497F-AC0C-F798A25CF170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6CB7C5-FCAC-4DA9-AF1C-2A167C87038A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6ABFC6CB-095B-4185-B39D-046E00DEABE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6ABFC6CB-095B-4185-B39D-046E00DEABE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Timbrado" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,29 @@
     <sheet name="TipoOtroPago" sheetId="4" r:id="rId4"/>
     <sheet name="TipoIncapacidad" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="231">
   <si>
     <t>RFC PATRONAL:</t>
   </si>
@@ -717,22 +729,22 @@
     <t>c_TipoIncapacidad</t>
   </si>
   <si>
-    <t>Riesgo de trabajo.</t>
-  </si>
-  <si>
-    <t>Enfermedad en general.</t>
-  </si>
-  <si>
-    <t>Maternidad.</t>
-  </si>
-  <si>
     <t>04</t>
   </si>
   <si>
-    <t>Licencia por cuidados médicos de hijos diagnosticados con cáncer.</t>
-  </si>
-  <si>
-    <t>No.Empleado</t>
+    <t>No. Empleado</t>
+  </si>
+  <si>
+    <t>Riesgo de trabajo</t>
+  </si>
+  <si>
+    <t>Enfermedad en general</t>
+  </si>
+  <si>
+    <t>Maternidad</t>
+  </si>
+  <si>
+    <t>Licencia por cuidados médicos de hijos diagnosticados con cáncer</t>
   </si>
 </sst>
 </file>
@@ -745,7 +757,7 @@
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="167" formatCode="00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -808,6 +820,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -841,7 +861,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -944,12 +964,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
@@ -1056,20 +1096,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -1077,9 +1105,6 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1094,27 +1119,67 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1446,110 +1511,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41371BBB-4714-4DEA-AB6C-BE84DA670BD5}">
-  <dimension ref="A2:X28"/>
+  <dimension ref="A2:Y41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
     <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="20" style="1" customWidth="1"/>
     <col min="7" max="7" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="1"/>
-    <col min="10" max="10" width="17.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16" style="1" customWidth="1"/>
-    <col min="12" max="12" width="32.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="11.42578125" style="1"/>
-    <col min="16" max="16" width="17.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" style="1" customWidth="1"/>
+    <col min="9" max="11" width="11.42578125" style="1"/>
+    <col min="12" max="12" width="17.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="32.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="11.42578125" style="1"/>
+    <col min="17" max="17" width="17.140625" style="1" customWidth="1"/>
     <col min="18" max="18" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="17.5703125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="12.28515625" style="1" customWidth="1"/>
     <col min="22" max="22" width="11.7109375" style="1" customWidth="1"/>
     <col min="23" max="23" width="20" style="1" customWidth="1"/>
     <col min="24" max="24" width="9.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="s">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="64"/>
+      <c r="B2" s="78"/>
       <c r="C2" s="43"/>
-      <c r="D2" s="49"/>
-      <c r="H2" s="67" t="s">
+      <c r="D2" s="45"/>
+      <c r="H2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="67"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="64" t="s">
+      <c r="I2" s="81"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="64"/>
-      <c r="D3" s="49"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="57" t="s">
+      <c r="B3" s="78"/>
+      <c r="D3" s="45"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="57"/>
+      <c r="B4" s="52"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="49"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" s="64" t="s">
+      <c r="D4" s="45"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="64"/>
-      <c r="D6" s="49"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="64" t="s">
+      <c r="B6" s="78"/>
+      <c r="D6" s="45"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="64"/>
-      <c r="D7" s="49"/>
+      <c r="B7" s="78"/>
+      <c r="D7" s="45"/>
       <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="D8" s="49"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="64" t="s">
+      <c r="B8" s="52"/>
+      <c r="D8" s="45"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A9" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="64"/>
-      <c r="D9" s="49"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="64" t="s">
+      <c r="B9" s="78"/>
+      <c r="D9" s="45"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="64"/>
+      <c r="B10" s="78"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="3"/>
+      <c r="D10" s="46"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -1557,15 +1625,15 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="57" t="s">
+      <c r="M10" s="3"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A11" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="57"/>
+      <c r="B11" s="52"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="3"/>
+      <c r="D11" s="46"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -1573,418 +1641,518 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="65" t="s">
+      <c r="M11" s="3"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A12" s="79" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="65"/>
-      <c r="D12" s="49"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A13" s="52"/>
-      <c r="B13" s="52"/>
-      <c r="D13" s="51"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E14" s="62" t="s">
+      <c r="B12" s="79"/>
+      <c r="D12" s="45"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A13" s="48"/>
+      <c r="B13" s="48"/>
+      <c r="D13" s="47"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="E14" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="62"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="62"/>
-      <c r="I14" s="62"/>
-      <c r="J14" s="62" t="s">
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="58"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="K14" s="62"/>
-      <c r="L14" s="62"/>
-      <c r="M14" s="62"/>
-    </row>
-    <row r="15" spans="1:24" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="66" t="s">
+      <c r="M14" s="77"/>
+      <c r="N14" s="77"/>
+    </row>
+    <row r="15" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="62" t="s">
+      <c r="B15" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="62" t="s">
+      <c r="D15" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="46" t="s">
+      <c r="E15" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="46" t="s">
+      <c r="F15" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="G15" s="46" t="s">
+      <c r="G15" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="44" t="s">
+      <c r="H15" s="65"/>
+      <c r="I15" s="65"/>
+      <c r="J15" s="58"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="K15" s="44" t="s">
-        <v>30</v>
-      </c>
-      <c r="L15" s="44" t="s">
+      <c r="M15" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="M15" s="45"/>
-      <c r="P15" s="63" t="s">
+      <c r="N15" s="69"/>
+      <c r="Q15" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="Q15" s="63"/>
-      <c r="R15" s="63"/>
-      <c r="S15" s="63"/>
-      <c r="T15" s="61"/>
-      <c r="U15" s="63" t="s">
+      <c r="R15" s="82"/>
+      <c r="S15" s="82"/>
+      <c r="T15" s="58"/>
+      <c r="U15" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="V15" s="63"/>
-      <c r="W15" s="63"/>
-      <c r="X15" s="63"/>
-    </row>
-    <row r="16" spans="1:24" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="66"/>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="46" t="s">
+      <c r="V15" s="75"/>
+      <c r="W15" s="75"/>
+      <c r="X15" s="76"/>
+    </row>
+    <row r="16" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="80"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="53" t="s">
+      <c r="F16" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="53" t="s">
+      <c r="G16" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="53" t="s">
+      <c r="H16" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="53" t="s">
+      <c r="I16" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="J16" s="46" t="s">
+      <c r="J16" s="58"/>
+      <c r="K16" s="70" t="s">
+        <v>9</v>
+      </c>
+      <c r="L16" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="K16" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="53" t="s">
+      <c r="M16" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="M16" s="53" t="s">
+      <c r="N16" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="O16" s="56" t="s">
+      <c r="P16" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="P16" s="48" t="s">
+      <c r="Q16" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="Q16" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="53" t="s">
+      <c r="R16" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="S16" s="53" t="s">
+      <c r="S16" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="T16" s="61"/>
-      <c r="U16" s="53" t="s">
-        <v>230</v>
-      </c>
-      <c r="V16" s="53" t="s">
+      <c r="T16" s="58"/>
+      <c r="U16" s="55" t="s">
+        <v>226</v>
+      </c>
+      <c r="V16" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="W16" s="53" t="s">
+      <c r="W16" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="X16" s="53" t="s">
+      <c r="X16" s="55" t="s">
         <v>23</v>
       </c>
+      <c r="Y16" s="64"/>
     </row>
     <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="50"/>
-      <c r="B17" s="50"/>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="50"/>
-      <c r="L17" s="50"/>
-      <c r="M17" s="50"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="50"/>
-      <c r="P17" s="50"/>
-      <c r="Q17" s="50"/>
-      <c r="R17" s="50"/>
-      <c r="S17" s="50"/>
-      <c r="T17" s="60"/>
-      <c r="U17" s="50"/>
-      <c r="V17" s="50"/>
-      <c r="W17" s="50"/>
-      <c r="X17" s="50"/>
+      <c r="A17" s="46"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="68"/>
+      <c r="K17" s="74"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="46"/>
+      <c r="N17" s="59"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="46"/>
+      <c r="Q17" s="46"/>
+      <c r="R17" s="46"/>
+      <c r="S17" s="59"/>
+      <c r="T17" s="57"/>
+      <c r="U17" s="46"/>
+      <c r="V17" s="46"/>
+      <c r="W17" s="46"/>
+      <c r="X17" s="59"/>
     </row>
     <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
-      <c r="B18" s="50"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="50"/>
-      <c r="M18" s="50"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="50"/>
-      <c r="P18" s="50"/>
-      <c r="Q18" s="50"/>
-      <c r="R18" s="50"/>
-      <c r="S18" s="50"/>
-      <c r="T18" s="60"/>
-      <c r="U18" s="50"/>
-      <c r="V18" s="50"/>
-      <c r="W18" s="50"/>
-      <c r="X18" s="50"/>
+      <c r="A18" s="46"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="59"/>
+      <c r="I18" s="59"/>
+      <c r="J18" s="68"/>
+      <c r="K18" s="73"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="59"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="46"/>
+      <c r="R18" s="46"/>
+      <c r="S18" s="59"/>
+      <c r="T18" s="57"/>
+      <c r="U18" s="46"/>
+      <c r="V18" s="46"/>
+      <c r="W18" s="46"/>
+      <c r="X18" s="59"/>
     </row>
     <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="Q19" s="50"/>
-      <c r="R19" s="50"/>
-      <c r="S19" s="50"/>
-      <c r="T19" s="60"/>
-      <c r="U19" s="50"/>
-      <c r="V19" s="50"/>
-      <c r="W19" s="50"/>
-      <c r="X19" s="50"/>
-    </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
-      <c r="B20" s="50"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="50"/>
+      <c r="A19" s="46"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="59"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="68"/>
+      <c r="K19" s="71"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="59"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="46"/>
+      <c r="R19" s="46"/>
+      <c r="S19" s="59"/>
+      <c r="T19" s="57"/>
+      <c r="U19" s="46"/>
+      <c r="V19" s="46"/>
+      <c r="W19" s="46"/>
+      <c r="X19" s="59"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A20" s="45"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
       <c r="G20" s="50"/>
-      <c r="H20" s="50"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="50"/>
-      <c r="K20" s="50"/>
-      <c r="L20" s="50"/>
-      <c r="M20" s="50"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="50"/>
-      <c r="P20" s="50"/>
-      <c r="Q20" s="50"/>
-      <c r="R20" s="50"/>
-      <c r="S20" s="50"/>
-      <c r="T20" s="60"/>
-      <c r="U20" s="50"/>
-      <c r="V20" s="50"/>
-      <c r="W20" s="50"/>
-      <c r="X20" s="50"/>
-    </row>
-    <row r="21" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="50"/>
-      <c r="B21" s="50"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
+      <c r="H20" s="60"/>
+      <c r="I20" s="60"/>
+      <c r="J20" s="68"/>
+      <c r="K20" s="72"/>
+      <c r="L20" s="49"/>
+      <c r="M20" s="45"/>
+      <c r="N20" s="60"/>
+      <c r="P20" s="45"/>
+      <c r="Q20" s="46"/>
+      <c r="R20" s="45"/>
+      <c r="S20" s="60"/>
+      <c r="T20" s="57"/>
+      <c r="U20" s="46"/>
+      <c r="V20" s="45"/>
+      <c r="W20" s="46"/>
+      <c r="X20" s="60"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A21" s="45"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
       <c r="G21" s="50"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="50"/>
-      <c r="K21" s="50"/>
-      <c r="L21" s="50"/>
-      <c r="M21" s="50"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="50"/>
-      <c r="P21" s="50"/>
-      <c r="Q21" s="50"/>
-      <c r="R21" s="50"/>
-      <c r="S21" s="50"/>
-      <c r="T21" s="60"/>
-      <c r="U21" s="50"/>
-      <c r="V21" s="50"/>
-      <c r="W21" s="50"/>
-      <c r="X21" s="50"/>
+      <c r="H21" s="60"/>
+      <c r="I21" s="60"/>
+      <c r="J21" s="68"/>
+      <c r="K21" s="72"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="60"/>
+      <c r="P21" s="45"/>
+      <c r="Q21" s="46"/>
+      <c r="R21" s="45"/>
+      <c r="S21" s="60"/>
+      <c r="T21" s="57"/>
+      <c r="U21" s="46"/>
+      <c r="V21" s="45"/>
+      <c r="W21" s="46"/>
+      <c r="X21" s="60"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A22" s="49"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="49"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="50"/>
-      <c r="K22" s="49"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="50"/>
+      <c r="H22" s="60"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="68"/>
+      <c r="K22" s="72"/>
       <c r="L22" s="49"/>
-      <c r="M22" s="49"/>
-      <c r="O22" s="49"/>
-      <c r="P22" s="49"/>
-      <c r="Q22" s="49"/>
-      <c r="R22" s="49"/>
-      <c r="S22" s="49"/>
-      <c r="T22" s="60"/>
-      <c r="U22" s="49"/>
-      <c r="V22" s="49"/>
-      <c r="W22" s="49"/>
-      <c r="X22" s="49"/>
+      <c r="M22" s="46"/>
+      <c r="N22" s="60"/>
+      <c r="P22" s="45"/>
+      <c r="Q22" s="46"/>
+      <c r="R22" s="45"/>
+      <c r="S22" s="60"/>
+      <c r="T22" s="57"/>
+      <c r="U22" s="46"/>
+      <c r="V22" s="45"/>
+      <c r="W22" s="46"/>
+      <c r="X22" s="60"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A23" s="49"/>
-      <c r="B23" s="50"/>
-      <c r="C23" s="50"/>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="50"/>
-      <c r="M23" s="49"/>
-      <c r="O23" s="49"/>
-      <c r="P23" s="49"/>
-      <c r="Q23" s="49"/>
-      <c r="R23" s="49"/>
-      <c r="S23" s="49"/>
-      <c r="T23" s="60"/>
-      <c r="U23" s="49"/>
-      <c r="V23" s="49"/>
-      <c r="W23" s="49"/>
-      <c r="X23" s="49"/>
+      <c r="A23" s="45"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
+      <c r="J23" s="68"/>
+      <c r="K23" s="72"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="60"/>
+      <c r="P23" s="45"/>
+      <c r="Q23" s="46"/>
+      <c r="R23" s="45"/>
+      <c r="S23" s="60"/>
+      <c r="T23" s="57"/>
+      <c r="U23" s="46"/>
+      <c r="V23" s="45"/>
+      <c r="W23" s="46"/>
+      <c r="X23" s="60"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A24" s="49"/>
-      <c r="B24" s="50"/>
-      <c r="C24" s="50"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="50"/>
-      <c r="M24" s="49"/>
-      <c r="O24" s="49"/>
-      <c r="P24" s="49"/>
-      <c r="Q24" s="49"/>
-      <c r="R24" s="49"/>
-      <c r="S24" s="49"/>
-      <c r="T24" s="60"/>
-      <c r="U24" s="49"/>
-      <c r="V24" s="49"/>
-      <c r="W24" s="49"/>
-      <c r="X24" s="49"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="61"/>
+      <c r="K24" s="61"/>
+      <c r="L24" s="49"/>
+      <c r="N24" s="61"/>
+      <c r="P24" s="45"/>
+      <c r="Q24" s="46"/>
+      <c r="R24" s="45"/>
+      <c r="S24" s="60"/>
+      <c r="T24" s="57"/>
+      <c r="U24" s="46"/>
+      <c r="V24" s="45"/>
+      <c r="W24" s="46"/>
+      <c r="X24" s="60"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A25" s="49"/>
-      <c r="B25" s="50"/>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="55"/>
-      <c r="M25" s="49"/>
-      <c r="O25" s="49"/>
-      <c r="P25" s="49"/>
-      <c r="Q25" s="49"/>
-      <c r="R25" s="49"/>
-      <c r="S25" s="49"/>
-      <c r="T25" s="60"/>
-      <c r="U25" s="49"/>
-      <c r="V25" s="49"/>
-      <c r="W25" s="49"/>
-      <c r="X25" s="49"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
-      <c r="G26" s="47"/>
-      <c r="O26" s="49"/>
-      <c r="P26" s="49"/>
-      <c r="Q26" s="49"/>
-      <c r="R26" s="49"/>
-      <c r="S26" s="49"/>
-      <c r="T26" s="60"/>
-      <c r="U26" s="49"/>
-      <c r="V26" s="49"/>
-      <c r="W26" s="49"/>
-      <c r="X26" s="49"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="3"/>
+      <c r="X26" s="3"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="G27" s="47"/>
+      <c r="H27" s="61"/>
+      <c r="I27" s="61"/>
+      <c r="J27" s="61"/>
+      <c r="K27" s="61"/>
+      <c r="N27" s="61"/>
+      <c r="S27" s="61"/>
+      <c r="V27" s="61"/>
+      <c r="X27" s="61"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="G28" s="47"/>
+      <c r="H28" s="61"/>
+      <c r="I28" s="61"/>
+      <c r="J28" s="61"/>
+      <c r="K28" s="61"/>
+      <c r="N28" s="61"/>
+      <c r="S28" s="61"/>
+      <c r="V28" s="61"/>
+      <c r="X28" s="61"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="H29" s="61"/>
+      <c r="I29" s="61"/>
+      <c r="J29" s="61"/>
+      <c r="K29" s="61"/>
+      <c r="N29" s="61"/>
+      <c r="S29" s="61"/>
+      <c r="V29" s="61"/>
+      <c r="X29" s="61"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="H30" s="61"/>
+      <c r="I30" s="61"/>
+      <c r="J30" s="61"/>
+      <c r="K30" s="61"/>
+      <c r="N30" s="61"/>
+      <c r="S30" s="62"/>
+      <c r="V30" s="61"/>
+      <c r="X30" s="61"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="H31" s="61"/>
+      <c r="I31" s="61"/>
+      <c r="J31" s="61"/>
+      <c r="K31" s="61"/>
+      <c r="N31" s="61"/>
+      <c r="S31" s="61"/>
+      <c r="V31" s="61"/>
+      <c r="X31" s="61"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="H32" s="61"/>
+      <c r="I32" s="61"/>
+      <c r="J32" s="61"/>
+      <c r="K32" s="61"/>
+      <c r="N32" s="61"/>
+      <c r="S32" s="61"/>
+      <c r="V32" s="61"/>
+      <c r="X32" s="61"/>
+    </row>
+    <row r="33" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H33" s="61"/>
+      <c r="I33" s="61"/>
+      <c r="J33" s="61"/>
+      <c r="K33" s="61"/>
+      <c r="N33" s="61"/>
+      <c r="S33" s="61"/>
+      <c r="V33" s="61"/>
+      <c r="X33" s="61"/>
+    </row>
+    <row r="34" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H34" s="61"/>
+      <c r="I34" s="61"/>
+      <c r="J34" s="61"/>
+      <c r="K34" s="61"/>
+      <c r="N34" s="61"/>
+      <c r="X34" s="61"/>
+    </row>
+    <row r="35" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H35" s="61"/>
+      <c r="I35" s="61"/>
+      <c r="J35" s="61"/>
+      <c r="K35" s="61"/>
+      <c r="N35" s="61"/>
+      <c r="X35" s="61"/>
+    </row>
+    <row r="36" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H36" s="61"/>
+      <c r="I36" s="61"/>
+      <c r="J36" s="61"/>
+      <c r="K36" s="61"/>
+      <c r="X36" s="61"/>
+    </row>
+    <row r="37" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H37" s="61"/>
+      <c r="I37" s="61"/>
+      <c r="J37" s="61"/>
+      <c r="K37" s="61"/>
+      <c r="X37" s="61"/>
+    </row>
+    <row r="38" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H38" s="61"/>
+      <c r="I38" s="61"/>
+      <c r="J38" s="61"/>
+      <c r="K38" s="61"/>
+    </row>
+    <row r="39" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H39" s="61"/>
+      <c r="I39" s="61"/>
+      <c r="J39" s="61"/>
+      <c r="K39" s="61"/>
+    </row>
+    <row r="40" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H40" s="61"/>
+      <c r="I40" s="61"/>
+      <c r="J40" s="61"/>
+      <c r="K40" s="61"/>
+    </row>
+    <row r="41" spans="8:24" x14ac:dyDescent="0.25">
+      <c r="H41" s="61"/>
+      <c r="I41" s="61"/>
+      <c r="J41" s="61"/>
+      <c r="K41" s="61"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="16">
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="E14:I14"/>
-    <mergeCell ref="J14:M14"/>
-    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="Q15:S15"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="U15:X15"/>
     <mergeCell ref="D15:D16"/>
-    <mergeCell ref="U15:X15"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A15:A16"/>
@@ -1992,7 +2160,7 @@
     <mergeCell ref="C15:C16"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6" xr:uid="{FB64CB1D-A4B2-4312-B0B3-4AE10CFD0BFA}">
       <formula1>"O,E"</formula1>
     </dataValidation>
@@ -2002,56 +2170,50 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C13" xr:uid="{9B35E0F7-3637-464B-B327-42D6159FCD3B}">
       <formula1>"IP, IF, IM"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6" xr:uid="{74D94BD4-970F-4B71-BB34-914D442E1749}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6" xr:uid="{9AB734E0-3220-4188-B39F-42F1D0A44583}">
       <formula1>"Nómina Ordinaria,Nómina Extraordinaria"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11" xr:uid="{E59F2988-4A54-46B5-9EB6-8B7641BBE687}">
+      <formula1>"Diario,Semanal,Catorcenal,Quincenal,Mensual,Bimestral,Unidad obra,Comisión,Precio alzado,Decenal,Otra Periodicidad"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D12" xr:uid="{6E8AB270-BD12-476D-A0FF-62B00D3A8132}">
+      <formula1>"Ingresos propios,Ingresos federales,Ingresos mixtos"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0511DD22-8215-43C6-A69E-5DAC5F5622D6}">
-          <x14:formula1>
-            <xm:f>TipoOtroPago!$A$6:$A$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>Q17 P18:P19</xm:sqref>
-        </x14:dataValidation>
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2D52521A-962B-40BB-89D2-8CB7925AF974}">
           <x14:formula1>
-            <xm:f>TipoOtroPago!$B$6:$B$15</xm:f>
+            <xm:f>TipoOtroPago!$F$6:$F$15</xm:f>
           </x14:formula1>
-          <xm:sqref>P17</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A6D12201-A78E-48A1-9176-B701CDCF4A5B}">
-          <x14:formula1>
-            <xm:f>Percepciones!$A$6:$A$49</xm:f>
-          </x14:formula1>
-          <xm:sqref>F17</xm:sqref>
+          <xm:sqref>Q17:Q24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E1BF81AA-AC21-476C-8F65-C86B9A11CE23}">
           <x14:formula1>
             <xm:f>Percepciones!$B$6:$B$49</xm:f>
           </x14:formula1>
-          <xm:sqref>E17</xm:sqref>
+          <xm:sqref>E17:E23</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C7FD529D-EBD1-44CB-A072-C49051014090}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56F2ED0B-3E68-4A97-A768-6C850C82DA62}">
           <x14:formula1>
-            <xm:f>Deducciones!$B$6:$B$112</xm:f>
+            <xm:f>TipoIncapacidad!$F$6:$F$9</xm:f>
           </x14:formula1>
-          <xm:sqref>J17</xm:sqref>
+          <xm:sqref>W17:W24</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F113C487-ADBA-41BE-BC29-CA1C80CF4B1D}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{527D78B9-3CFD-41EB-B65D-D922748B021C}">
           <x14:formula1>
-            <xm:f>Deducciones!$A$6:$A$112</xm:f>
+            <xm:f>Percepciones!$F$6:$F$49</xm:f>
           </x14:formula1>
-          <xm:sqref>K17</xm:sqref>
+          <xm:sqref>F17:F23</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{90E78F9B-A7A2-4F7F-9DB0-1F1207EE64AD}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0F30A284-2059-462B-A411-B81C0FC0D032}">
           <x14:formula1>
-            <xm:f>TipoIncapacidad!$B$6:$B$9</xm:f>
+            <xm:f>Deducciones!$F$6:$F$112</xm:f>
           </x14:formula1>
-          <xm:sqref>W17</xm:sqref>
+          <xm:sqref>L17:L24</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2061,22 +2223,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE09CAF-264C-4767-9880-4BE0C5984EDC}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="88.7109375" style="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="68" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="68"/>
+      <c r="B1" s="83"/>
       <c r="C1" s="5"/>
       <c r="D1" s="6"/>
     </row>
-    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>35</v>
       </c>
@@ -2088,7 +2250,7 @@
       </c>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -2100,13 +2262,13 @@
       </c>
       <c r="D3" s="5"/>
     </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="19"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
     </row>
-    <row r="5" spans="1:4" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>38</v>
       </c>
@@ -2120,7 +2282,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>1</v>
       </c>
@@ -2131,8 +2293,12 @@
         <v>42675</v>
       </c>
       <c r="D6" s="15"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" t="str">
+        <f>VALUE(A6) &amp; " - " &amp; B6</f>
+        <v>1 - Sueldos, Salarios  Rayas y Jornales</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="13">
         <v>2</v>
       </c>
@@ -2143,8 +2309,12 @@
         <v>42675</v>
       </c>
       <c r="D7" s="15"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" t="str">
+        <f t="shared" ref="F7:F49" si="0">VALUE(A7) &amp; " - " &amp; B7</f>
+        <v>2 - Gratificación Anual (Aguinaldo)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>3</v>
       </c>
@@ -2155,8 +2325,12 @@
         <v>42675</v>
       </c>
       <c r="D8" s="15"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>3 - Participación de los Trabajadores en las Utilidades PTU</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="13">
         <v>4</v>
       </c>
@@ -2167,8 +2341,12 @@
         <v>42675</v>
       </c>
       <c r="D9" s="15"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>4 - Reembolso de Gastos Médicos Dentales y Hospitalarios</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>5</v>
       </c>
@@ -2179,8 +2357,12 @@
         <v>42675</v>
       </c>
       <c r="D10" s="15"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>5 - Fondo de Ahorro</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="13">
         <v>6</v>
       </c>
@@ -2191,8 +2373,12 @@
         <v>42675</v>
       </c>
       <c r="D11" s="15"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>6 - Caja de ahorro</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>9</v>
       </c>
@@ -2203,8 +2389,12 @@
         <v>42675</v>
       </c>
       <c r="D12" s="15"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>9 - Contribuciones a Cargo del Trabajador Pagadas por el Patrón</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13">
         <v>10</v>
       </c>
@@ -2215,8 +2405,12 @@
         <v>42675</v>
       </c>
       <c r="D13" s="15"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>10 - Premios por puntualidad</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>11</v>
       </c>
@@ -2227,8 +2421,12 @@
         <v>42675</v>
       </c>
       <c r="D14" s="15"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>11 - Prima de Seguro de vida</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="13">
         <v>12</v>
       </c>
@@ -2239,8 +2437,12 @@
         <v>42675</v>
       </c>
       <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>12 - Seguro de Gastos Médicos Mayores</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
         <v>13</v>
       </c>
@@ -2251,8 +2453,12 @@
         <v>42675</v>
       </c>
       <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>13 - Cuotas Sindicales Pagadas por el Patrón</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="13">
         <v>14</v>
       </c>
@@ -2263,8 +2469,12 @@
         <v>42675</v>
       </c>
       <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" t="str">
+        <f t="shared" si="0"/>
+        <v>14 - Subsidios por incapacidad</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="13">
         <v>15</v>
       </c>
@@ -2275,8 +2485,12 @@
         <v>42675</v>
       </c>
       <c r="D18" s="15"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" t="str">
+        <f t="shared" si="0"/>
+        <v>15 - Becas para trabajadores y/o hijos</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="13">
         <v>19</v>
       </c>
@@ -2287,8 +2501,12 @@
         <v>42675</v>
       </c>
       <c r="D19" s="15"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F19" t="str">
+        <f t="shared" si="0"/>
+        <v>19 - Horas extra</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="13">
         <v>20</v>
       </c>
@@ -2299,8 +2517,12 @@
         <v>42675</v>
       </c>
       <c r="D20" s="15"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F20" t="str">
+        <f t="shared" si="0"/>
+        <v>20 - Prima dominical</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="13">
         <v>21</v>
       </c>
@@ -2311,8 +2533,12 @@
         <v>42675</v>
       </c>
       <c r="D21" s="15"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F21" t="str">
+        <f t="shared" si="0"/>
+        <v>21 - Prima vacacional</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="13">
         <v>22</v>
       </c>
@@ -2323,8 +2549,12 @@
         <v>42675</v>
       </c>
       <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F22" t="str">
+        <f t="shared" si="0"/>
+        <v>22 - Prima por antigüedad</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="13">
         <v>23</v>
       </c>
@@ -2335,8 +2565,12 @@
         <v>42675</v>
       </c>
       <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F23" t="str">
+        <f t="shared" si="0"/>
+        <v>23 - Pagos por separación</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="13">
         <v>24</v>
       </c>
@@ -2347,8 +2581,12 @@
         <v>42675</v>
       </c>
       <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F24" t="str">
+        <f t="shared" si="0"/>
+        <v>24 - Seguro de retiro</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="13">
         <v>25</v>
       </c>
@@ -2359,8 +2597,12 @@
         <v>42675</v>
       </c>
       <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F25" t="str">
+        <f t="shared" si="0"/>
+        <v>25 - Indemnizaciones</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>26</v>
       </c>
@@ -2371,8 +2613,12 @@
         <v>42675</v>
       </c>
       <c r="D26" s="15"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F26" t="str">
+        <f t="shared" si="0"/>
+        <v>26 - Reembolso por funeral</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="13">
         <v>27</v>
       </c>
@@ -2383,8 +2629,12 @@
         <v>42675</v>
       </c>
       <c r="D27" s="15"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F27" t="str">
+        <f t="shared" si="0"/>
+        <v>27 - Cuotas de seguridad social pagadas por el patrón</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="13">
         <v>28</v>
       </c>
@@ -2395,8 +2645,12 @@
         <v>42675</v>
       </c>
       <c r="D28" s="15"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F28" t="str">
+        <f t="shared" si="0"/>
+        <v>28 - Comisiones</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="13">
         <v>29</v>
       </c>
@@ -2407,8 +2661,12 @@
         <v>42675</v>
       </c>
       <c r="D29" s="15"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F29" t="str">
+        <f t="shared" si="0"/>
+        <v>29 - Vales de despensa</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="13">
         <v>30</v>
       </c>
@@ -2419,8 +2677,12 @@
         <v>42675</v>
       </c>
       <c r="D30" s="15"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F30" t="str">
+        <f t="shared" si="0"/>
+        <v>30 - Vales de restaurante</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="13">
         <v>31</v>
       </c>
@@ -2431,8 +2693,12 @@
         <v>42675</v>
       </c>
       <c r="D31" s="15"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F31" t="str">
+        <f t="shared" si="0"/>
+        <v>31 - Vales de gasolina</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="13">
         <v>32</v>
       </c>
@@ -2443,8 +2709,12 @@
         <v>42675</v>
       </c>
       <c r="D32" s="15"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F32" t="str">
+        <f t="shared" si="0"/>
+        <v>32 - Vales de ropa</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="13">
         <v>33</v>
       </c>
@@ -2455,8 +2725,12 @@
         <v>42675</v>
       </c>
       <c r="D33" s="15"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F33" t="str">
+        <f t="shared" si="0"/>
+        <v>33 - Ayuda para renta</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="13">
         <v>34</v>
       </c>
@@ -2467,8 +2741,12 @@
         <v>42675</v>
       </c>
       <c r="D34" s="15"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F34" t="str">
+        <f t="shared" si="0"/>
+        <v>34 - Ayuda para artículos escolares</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="13">
         <v>35</v>
       </c>
@@ -2479,8 +2757,12 @@
         <v>42675</v>
       </c>
       <c r="D35" s="15"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F35" t="str">
+        <f t="shared" si="0"/>
+        <v>35 - Ayuda para anteojos</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="13">
         <v>36</v>
       </c>
@@ -2491,8 +2773,12 @@
         <v>42675</v>
       </c>
       <c r="D36" s="15"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F36" t="str">
+        <f t="shared" si="0"/>
+        <v>36 - Ayuda para transporte</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="13">
         <v>37</v>
       </c>
@@ -2503,8 +2789,12 @@
         <v>42675</v>
       </c>
       <c r="D37" s="15"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F37" t="str">
+        <f t="shared" si="0"/>
+        <v>37 - Ayuda para gastos de funeral</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="13">
         <v>38</v>
       </c>
@@ -2515,8 +2805,12 @@
         <v>42675</v>
       </c>
       <c r="D38" s="15"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F38" t="str">
+        <f t="shared" si="0"/>
+        <v>38 - Otros ingresos por salarios</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="13">
         <v>39</v>
       </c>
@@ -2527,8 +2821,12 @@
         <v>42675</v>
       </c>
       <c r="D39" s="15"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F39" t="str">
+        <f t="shared" si="0"/>
+        <v>39 - Jubilaciones, pensiones o haberes de retiro</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="13">
         <v>44</v>
       </c>
@@ -2539,8 +2837,12 @@
         <v>42675</v>
       </c>
       <c r="D40" s="15"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F40" t="str">
+        <f t="shared" si="0"/>
+        <v>44 - Jubilaciones, pensiones o haberes de retiro en parcialidades</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="13">
         <v>45</v>
       </c>
@@ -2551,8 +2853,12 @@
         <v>42675</v>
       </c>
       <c r="D41" s="15"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F41" t="str">
+        <f t="shared" si="0"/>
+        <v>45 - Ingresos en acciones o títulos valor que representan bienes</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="13">
         <v>46</v>
       </c>
@@ -2563,8 +2869,12 @@
         <v>42675</v>
       </c>
       <c r="D42" s="15"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F42" t="str">
+        <f t="shared" si="0"/>
+        <v>46 - Ingresos asimilados a salarios</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="13">
         <v>47</v>
       </c>
@@ -2575,8 +2885,12 @@
         <v>42675</v>
       </c>
       <c r="D43" s="15"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F43" t="str">
+        <f t="shared" si="0"/>
+        <v>47 - Alimentación diferentes a los establecidos en el Art 94 último párrafo LISR</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="13">
         <v>48</v>
       </c>
@@ -2587,8 +2901,12 @@
         <v>42675</v>
       </c>
       <c r="D44" s="15"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F44" t="str">
+        <f t="shared" si="0"/>
+        <v>48 - Habitación</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="13">
         <v>49</v>
       </c>
@@ -2599,8 +2917,12 @@
         <v>42675</v>
       </c>
       <c r="D45" s="15"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F45" t="str">
+        <f t="shared" si="0"/>
+        <v>49 - Premios por asistencia</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="13">
         <v>50</v>
       </c>
@@ -2611,8 +2933,12 @@
         <v>42741</v>
       </c>
       <c r="D46" s="15"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F46" t="str">
+        <f t="shared" si="0"/>
+        <v>50 - Viáticos</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="13">
         <v>51</v>
       </c>
@@ -2623,8 +2949,12 @@
         <v>43388</v>
       </c>
       <c r="D47" s="16"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F47" t="str">
+        <f t="shared" si="0"/>
+        <v>51 - Pagos por gratificaciones, primas, compensaciones, recompensas u otros a extrabajadores derivados de jubilación en parcialidades</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="13">
         <v>52</v>
       </c>
@@ -2635,8 +2965,12 @@
         <v>43388</v>
       </c>
       <c r="D48" s="16"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F48" t="str">
+        <f t="shared" si="0"/>
+        <v>52 - Pagos que se realicen a extrabajadores que obtengan una jubilación en parcialidades derivados de la ejecución de resoluciones judicial o de un laudo</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="13">
         <v>53</v>
       </c>
@@ -2647,6 +2981,10 @@
         <v>43388</v>
       </c>
       <c r="D49" s="16"/>
+      <c r="F49" t="str">
+        <f t="shared" si="0"/>
+        <v>53 - Pagos que se realicen a extrabajadores que obtengan una jubilación en una sola exhibición derivados de la ejecución de resoluciones judicial o de un laudo</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2658,7 +2996,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F49D385A-5A19-4DDA-852E-80C232EFEC42}">
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -2667,16 +3005,16 @@
     <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="84" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="69"/>
+      <c r="B1" s="84"/>
       <c r="C1" s="19"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="71"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D1" s="85"/>
+      <c r="E1" s="86"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>35</v>
       </c>
@@ -2689,7 +3027,7 @@
       <c r="D2" s="19"/>
       <c r="E2" s="25"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="28">
         <v>4</v>
       </c>
@@ -2702,14 +3040,14 @@
       <c r="D3" s="19"/>
       <c r="E3" s="25"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="19"/>
       <c r="C4" s="30"/>
       <c r="D4" s="19"/>
       <c r="E4" s="19"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>86</v>
       </c>
@@ -2724,7 +3062,7 @@
       </c>
       <c r="E5" s="32"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <v>1</v>
       </c>
@@ -2736,8 +3074,12 @@
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="32"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" t="str">
+        <f>VALUE(A6) &amp; " - " &amp;B6</f>
+        <v>1 - Seguridad social</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <v>2</v>
       </c>
@@ -2749,8 +3091,12 @@
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="32"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" t="str">
+        <f t="shared" ref="F7:F70" si="0">VALUE(A7) &amp; " - " &amp;B7</f>
+        <v>2 - ISR</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <v>3</v>
       </c>
@@ -2762,8 +3108,12 @@
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="32"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>3 - Aportaciones a retiro, cesantía en edad avanzada y vejez.</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <v>4</v>
       </c>
@@ -2775,8 +3125,12 @@
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="32"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>4 - Otros</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <v>5</v>
       </c>
@@ -2788,8 +3142,12 @@
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="32"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>5 - Aportaciones a Fondo de vivienda</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <v>6</v>
       </c>
@@ -2801,8 +3159,12 @@
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="32"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>6 - Descuento por incapacidad</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <v>7</v>
       </c>
@@ -2814,8 +3176,12 @@
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="32"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>7 - Pensión alimenticia</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <v>8</v>
       </c>
@@ -2827,8 +3193,12 @@
       </c>
       <c r="D13" s="14"/>
       <c r="E13" s="32"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>8 - Renta</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <v>9</v>
       </c>
@@ -2840,8 +3210,12 @@
       </c>
       <c r="D14" s="14"/>
       <c r="E14" s="32"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>9 - Préstamos provenientes del Fondo Nacional de la Vivienda para los Trabajadores</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <v>10</v>
       </c>
@@ -2853,8 +3227,12 @@
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="32"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>10 - Pago por crédito de vivienda</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <v>11</v>
       </c>
@@ -2866,8 +3244,12 @@
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="32"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>11 - Pago de abonos INFONACOT</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <v>12</v>
       </c>
@@ -2879,8 +3261,12 @@
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="32"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" t="str">
+        <f t="shared" si="0"/>
+        <v>12 - Anticipo de salarios</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <v>13</v>
       </c>
@@ -2892,8 +3278,12 @@
       </c>
       <c r="D18" s="14"/>
       <c r="E18" s="32"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" t="str">
+        <f t="shared" si="0"/>
+        <v>13 - Pagos hechos con exceso al trabajador</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <v>14</v>
       </c>
@@ -2905,8 +3295,12 @@
       </c>
       <c r="D19" s="14"/>
       <c r="E19" s="32"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" t="str">
+        <f t="shared" si="0"/>
+        <v>14 - Errores</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <v>15</v>
       </c>
@@ -2918,8 +3312,12 @@
       </c>
       <c r="D20" s="14"/>
       <c r="E20" s="32"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" t="str">
+        <f t="shared" si="0"/>
+        <v>15 - Pérdidas</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <v>16</v>
       </c>
@@ -2931,8 +3329,12 @@
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="32"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" t="str">
+        <f t="shared" si="0"/>
+        <v>16 - Averías</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <v>17</v>
       </c>
@@ -2944,8 +3346,12 @@
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="32"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" t="str">
+        <f t="shared" si="0"/>
+        <v>17 - Adquisición de artículos producidos por la empresa o establecimiento</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <v>18</v>
       </c>
@@ -2957,8 +3363,12 @@
       </c>
       <c r="D23" s="14"/>
       <c r="E23" s="32"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" t="str">
+        <f t="shared" si="0"/>
+        <v>18 - Cuotas para la constitución y fomento de sociedades cooperativas y de cajas de ahorro</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <v>19</v>
       </c>
@@ -2970,8 +3380,12 @@
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="32"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" t="str">
+        <f t="shared" si="0"/>
+        <v>19 - Cuotas sindicales</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <v>20</v>
       </c>
@@ -2983,8 +3397,12 @@
       </c>
       <c r="D25" s="14"/>
       <c r="E25" s="32"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" t="str">
+        <f t="shared" si="0"/>
+        <v>20 - Ausencia (Ausentismo)</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <v>21</v>
       </c>
@@ -2996,8 +3414,12 @@
       </c>
       <c r="D26" s="14"/>
       <c r="E26" s="32"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" t="str">
+        <f t="shared" si="0"/>
+        <v>21 - Cuotas obrero patronales</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <v>22</v>
       </c>
@@ -3009,8 +3431,12 @@
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="19"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" t="str">
+        <f t="shared" si="0"/>
+        <v>22 - Impuestos Locales</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <v>23</v>
       </c>
@@ -3022,8 +3448,12 @@
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="19"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" t="str">
+        <f t="shared" si="0"/>
+        <v>23 - Aportaciones voluntarias</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="33">
         <v>24</v>
       </c>
@@ -3035,8 +3465,12 @@
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="19"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" t="str">
+        <f t="shared" si="0"/>
+        <v>24 - Ajuste en Gratificación Anual (Aguinaldo) Exento</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="33">
         <v>25</v>
       </c>
@@ -3048,8 +3482,12 @@
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="19"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" t="str">
+        <f t="shared" si="0"/>
+        <v>25 - Ajuste en Gratificación Anual (Aguinaldo) Gravado</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="33">
         <v>26</v>
       </c>
@@ -3061,8 +3499,12 @@
       </c>
       <c r="D31" s="14"/>
       <c r="E31" s="19"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" t="str">
+        <f t="shared" si="0"/>
+        <v>26 - Ajuste en Participación de los Trabajadores en las Utilidades PTU Exento</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="33">
         <v>27</v>
       </c>
@@ -3074,8 +3516,12 @@
       </c>
       <c r="D32" s="14"/>
       <c r="E32" s="19"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" t="str">
+        <f t="shared" si="0"/>
+        <v>27 - Ajuste en Participación de los Trabajadores en las Utilidades PTU Gravado</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="33">
         <v>28</v>
       </c>
@@ -3087,8 +3533,12 @@
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="19"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" t="str">
+        <f t="shared" si="0"/>
+        <v>28 - Ajuste en Reembolso de Gastos Médicos Dentales y Hospitalarios Exento</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="33">
         <v>29</v>
       </c>
@@ -3100,8 +3550,12 @@
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="19"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" t="str">
+        <f t="shared" si="0"/>
+        <v>29 - Ajuste en Fondo de ahorro Exento</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="33">
         <v>30</v>
       </c>
@@ -3113,8 +3567,12 @@
       </c>
       <c r="D35" s="14"/>
       <c r="E35" s="19"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" t="str">
+        <f t="shared" si="0"/>
+        <v>30 - Ajuste en Caja de ahorro Exento</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="33">
         <v>31</v>
       </c>
@@ -3126,8 +3584,12 @@
       </c>
       <c r="D36" s="14"/>
       <c r="E36" s="19"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" t="str">
+        <f t="shared" si="0"/>
+        <v>31 - Ajuste en Contribuciones a Cargo del Trabajador Pagadas por el Patrón Exento</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="33">
         <v>32</v>
       </c>
@@ -3139,8 +3601,12 @@
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="19"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" t="str">
+        <f t="shared" si="0"/>
+        <v>32 - Ajuste en Premios por puntualidad Gravado</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="33">
         <v>33</v>
       </c>
@@ -3152,8 +3618,12 @@
       </c>
       <c r="D38" s="14"/>
       <c r="E38" s="19"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" t="str">
+        <f t="shared" si="0"/>
+        <v>33 - Ajuste en Prima de Seguro de vida Exento</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="33">
         <v>34</v>
       </c>
@@ -3165,8 +3635,12 @@
       </c>
       <c r="D39" s="14"/>
       <c r="E39" s="19"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" t="str">
+        <f t="shared" si="0"/>
+        <v>34 - Ajuste en Seguro de Gastos Médicos Mayores Exento</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="33">
         <v>35</v>
       </c>
@@ -3178,8 +3652,12 @@
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="19"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" t="str">
+        <f t="shared" si="0"/>
+        <v>35 - Ajuste en Cuotas Sindicales Pagadas por el Patrón Exento</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="33">
         <v>36</v>
       </c>
@@ -3191,8 +3669,12 @@
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="19"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" t="str">
+        <f t="shared" si="0"/>
+        <v>36 - Ajuste en Subsidios por incapacidad Exento</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="33">
         <v>37</v>
       </c>
@@ -3204,8 +3686,12 @@
       </c>
       <c r="D42" s="14"/>
       <c r="E42" s="19"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" t="str">
+        <f t="shared" si="0"/>
+        <v>37 - Ajuste en Becas para trabajadores y/o hijos Exento</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="33">
         <v>38</v>
       </c>
@@ -3217,8 +3703,12 @@
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="19"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" t="str">
+        <f t="shared" si="0"/>
+        <v>38 - Ajuste en Horas extra Exento</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="33">
         <v>39</v>
       </c>
@@ -3230,8 +3720,12 @@
       </c>
       <c r="D44" s="14"/>
       <c r="E44" s="19"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" t="str">
+        <f t="shared" si="0"/>
+        <v>39 - Ajuste en Horas extra Gravado</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="33">
         <v>40</v>
       </c>
@@ -3243,8 +3737,12 @@
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="19"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" t="str">
+        <f t="shared" si="0"/>
+        <v>40 - Ajuste en Prima dominical Exento</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="33">
         <v>41</v>
       </c>
@@ -3256,8 +3754,12 @@
       </c>
       <c r="D46" s="14"/>
       <c r="E46" s="19"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" t="str">
+        <f t="shared" si="0"/>
+        <v>41 - Ajuste en Prima dominical Gravado</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="33">
         <v>42</v>
       </c>
@@ -3269,8 +3771,12 @@
       </c>
       <c r="D47" s="14"/>
       <c r="E47" s="19"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" t="str">
+        <f t="shared" si="0"/>
+        <v>42 - Ajuste en Prima vacacional Exento</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="33">
         <v>43</v>
       </c>
@@ -3282,8 +3788,12 @@
       </c>
       <c r="D48" s="14"/>
       <c r="E48" s="19"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" t="str">
+        <f t="shared" si="0"/>
+        <v>43 - Ajuste en Prima vacacional Gravado</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="33">
         <v>44</v>
       </c>
@@ -3295,8 +3805,12 @@
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="19"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" t="str">
+        <f t="shared" si="0"/>
+        <v>44 - Ajuste en Prima por antigüedad Exento</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="33">
         <v>45</v>
       </c>
@@ -3308,8 +3822,12 @@
       </c>
       <c r="D50" s="14"/>
       <c r="E50" s="19"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" t="str">
+        <f t="shared" si="0"/>
+        <v>45 - Ajuste en Prima por antigüedad Gravado</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="33">
         <v>46</v>
       </c>
@@ -3321,8 +3839,12 @@
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="19"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" t="str">
+        <f t="shared" si="0"/>
+        <v>46 - Ajuste en Pagos por separación Exento</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="33">
         <v>47</v>
       </c>
@@ -3334,8 +3856,12 @@
       </c>
       <c r="D52" s="14"/>
       <c r="E52" s="19"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" t="str">
+        <f t="shared" si="0"/>
+        <v>47 - Ajuste en Pagos por separación Gravado</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="33">
         <v>48</v>
       </c>
@@ -3347,8 +3873,12 @@
       </c>
       <c r="D53" s="14"/>
       <c r="E53" s="19"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" t="str">
+        <f t="shared" si="0"/>
+        <v>48 - Ajuste en Seguro de retiro Exento</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="33">
         <v>49</v>
       </c>
@@ -3360,8 +3890,12 @@
       </c>
       <c r="D54" s="14"/>
       <c r="E54" s="19"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" t="str">
+        <f t="shared" si="0"/>
+        <v>49 - Ajuste en Indemnizaciones Exento</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="33">
         <v>50</v>
       </c>
@@ -3373,8 +3907,12 @@
       </c>
       <c r="D55" s="14"/>
       <c r="E55" s="19"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" t="str">
+        <f t="shared" si="0"/>
+        <v>50 - Ajuste en Indemnizaciones Gravado</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="33">
         <v>51</v>
       </c>
@@ -3386,8 +3924,12 @@
       </c>
       <c r="D56" s="14"/>
       <c r="E56" s="19"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" t="str">
+        <f t="shared" si="0"/>
+        <v>51 - Ajuste en Reembolso por funeral Exento</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="33">
         <v>52</v>
       </c>
@@ -3399,8 +3941,12 @@
       </c>
       <c r="D57" s="14"/>
       <c r="E57" s="19"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" t="str">
+        <f t="shared" si="0"/>
+        <v>52 - Ajuste en Cuotas de seguridad social pagadas por el patrón Exento</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="33">
         <v>53</v>
       </c>
@@ -3412,8 +3958,12 @@
       </c>
       <c r="D58" s="14"/>
       <c r="E58" s="19"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" t="str">
+        <f t="shared" si="0"/>
+        <v>53 - Ajuste en Comisiones Gravado</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="33">
         <v>54</v>
       </c>
@@ -3425,8 +3975,12 @@
       </c>
       <c r="D59" s="14"/>
       <c r="E59" s="19"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" t="str">
+        <f t="shared" si="0"/>
+        <v>54 - Ajuste en Vales de despensa Exento</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="33">
         <v>55</v>
       </c>
@@ -3438,8 +3992,12 @@
       </c>
       <c r="D60" s="14"/>
       <c r="E60" s="19"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" t="str">
+        <f t="shared" si="0"/>
+        <v>55 - Ajuste en Vales de restaurante Exento</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="33">
         <v>56</v>
       </c>
@@ -3451,8 +4009,12 @@
       </c>
       <c r="D61" s="14"/>
       <c r="E61" s="19"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" t="str">
+        <f t="shared" si="0"/>
+        <v>56 - Ajuste en Vales de gasolina Exento</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="33">
         <v>57</v>
       </c>
@@ -3464,8 +4026,12 @@
       </c>
       <c r="D62" s="14"/>
       <c r="E62" s="19"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" t="str">
+        <f t="shared" si="0"/>
+        <v>57 - Ajuste en Vales de ropa Exento</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="33">
         <v>58</v>
       </c>
@@ -3477,8 +4043,12 @@
       </c>
       <c r="D63" s="14"/>
       <c r="E63" s="19"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" t="str">
+        <f t="shared" si="0"/>
+        <v>58 - Ajuste en Ayuda para renta Exento</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="33">
         <v>59</v>
       </c>
@@ -3490,8 +4060,12 @@
       </c>
       <c r="D64" s="14"/>
       <c r="E64" s="19"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" t="str">
+        <f t="shared" si="0"/>
+        <v>59 - Ajuste en Ayuda para artículos escolares Exento</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="33">
         <v>60</v>
       </c>
@@ -3503,8 +4077,12 @@
       </c>
       <c r="D65" s="14"/>
       <c r="E65" s="19"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" t="str">
+        <f t="shared" si="0"/>
+        <v>60 - Ajuste en Ayuda para anteojos Exento</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="33">
         <v>61</v>
       </c>
@@ -3516,8 +4094,12 @@
       </c>
       <c r="D66" s="14"/>
       <c r="E66" s="19"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" t="str">
+        <f t="shared" si="0"/>
+        <v>61 - Ajuste en Ayuda para transporte Exento</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="33">
         <v>62</v>
       </c>
@@ -3529,8 +4111,12 @@
       </c>
       <c r="D67" s="14"/>
       <c r="E67" s="19"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" t="str">
+        <f t="shared" si="0"/>
+        <v>62 - Ajuste en Ayuda para gastos de funeral Exento</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="33">
         <v>63</v>
       </c>
@@ -3542,8 +4128,12 @@
       </c>
       <c r="D68" s="14"/>
       <c r="E68" s="19"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" t="str">
+        <f t="shared" si="0"/>
+        <v>63 - Ajuste en Otros ingresos por salarios Exento</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="33">
         <v>64</v>
       </c>
@@ -3555,8 +4145,12 @@
       </c>
       <c r="D69" s="14"/>
       <c r="E69" s="19"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" t="str">
+        <f t="shared" si="0"/>
+        <v>64 - Ajuste en Otros ingresos por salarios Gravado</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="33">
         <v>65</v>
       </c>
@@ -3568,8 +4162,12 @@
       </c>
       <c r="D70" s="14"/>
       <c r="E70" s="19"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">65 - Ajuste en Jubilaciones, pensiones o haberes de retiro en una sola exhibición Exento </v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="33">
         <v>66</v>
       </c>
@@ -3581,8 +4179,12 @@
       </c>
       <c r="D71" s="14"/>
       <c r="E71" s="19"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" t="str">
+        <f t="shared" ref="F71:F112" si="1">VALUE(A71) &amp; " - " &amp;B71</f>
+        <v>66 - Ajuste en Jubilaciones, pensiones o haberes de retiro en una sola exhibición Gravado</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="33">
         <v>67</v>
       </c>
@@ -3594,8 +4196,12 @@
       </c>
       <c r="D72" s="14"/>
       <c r="E72" s="19"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" t="str">
+        <f t="shared" si="1"/>
+        <v>67 - Ajuste en Pagos por separación Acumulable</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="33">
         <v>68</v>
       </c>
@@ -3607,8 +4213,12 @@
       </c>
       <c r="D73" s="14"/>
       <c r="E73" s="19"/>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" t="str">
+        <f t="shared" si="1"/>
+        <v>68 - Ajuste en Pagos por separación No acumulable</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="33">
         <v>69</v>
       </c>
@@ -3620,8 +4230,12 @@
       </c>
       <c r="D74" s="14"/>
       <c r="E74" s="19"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" t="str">
+        <f t="shared" si="1"/>
+        <v>69 - Ajuste en Jubilaciones, pensiones o haberes de retiro en parcialidades Exento</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="33">
         <v>70</v>
       </c>
@@ -3633,8 +4247,12 @@
       </c>
       <c r="D75" s="14"/>
       <c r="E75" s="19"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" t="str">
+        <f t="shared" si="1"/>
+        <v>70 - Ajuste en Jubilaciones, pensiones o haberes de retiro en parcialidades Gravado</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="33">
         <v>71</v>
       </c>
@@ -3646,8 +4264,12 @@
       </c>
       <c r="D76" s="14"/>
       <c r="E76" s="19"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" t="str">
+        <f t="shared" si="1"/>
+        <v>71 - Ajuste en Subsidio para el empleo (efectivamente entregado al trabajador)</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="33">
         <v>72</v>
       </c>
@@ -3661,8 +4283,12 @@
         <v>43387</v>
       </c>
       <c r="E77" s="19"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" t="str">
+        <f t="shared" si="1"/>
+        <v>72 - Ajuste en Ingresos en acciones o títulos valor que representan bienes Exento</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="33">
         <v>73</v>
       </c>
@@ -3674,8 +4300,12 @@
       </c>
       <c r="D78" s="14"/>
       <c r="E78" s="19"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" t="str">
+        <f t="shared" si="1"/>
+        <v>73 - Ajuste en Ingresos en acciones o títulos valor que representan bienes Gravado</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="33">
         <v>74</v>
       </c>
@@ -3687,8 +4317,12 @@
       </c>
       <c r="D79" s="14"/>
       <c r="E79" s="19"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" t="str">
+        <f t="shared" si="1"/>
+        <v>74 - Ajuste en Alimentación Exento</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="33">
         <v>75</v>
       </c>
@@ -3700,8 +4334,12 @@
       </c>
       <c r="D80" s="14"/>
       <c r="E80" s="19"/>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" t="str">
+        <f t="shared" si="1"/>
+        <v>75 - Ajuste en Alimentación Gravado</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="33">
         <v>76</v>
       </c>
@@ -3713,8 +4351,12 @@
       </c>
       <c r="D81" s="14"/>
       <c r="E81" s="19"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" t="str">
+        <f t="shared" si="1"/>
+        <v>76 - Ajuste en Habitación Exento</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="33">
         <v>77</v>
       </c>
@@ -3726,8 +4368,12 @@
       </c>
       <c r="D82" s="14"/>
       <c r="E82" s="19"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82" t="str">
+        <f t="shared" si="1"/>
+        <v>77 - Ajuste en Habitación Gravado</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="33">
         <v>78</v>
       </c>
@@ -3739,8 +4385,12 @@
       </c>
       <c r="D83" s="14"/>
       <c r="E83" s="19"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83" t="str">
+        <f t="shared" si="1"/>
+        <v>78 - Ajuste en Premios por asistencia</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="33">
         <v>79</v>
       </c>
@@ -3752,8 +4402,12 @@
       </c>
       <c r="D84" s="14"/>
       <c r="E84" s="19"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84" t="str">
+        <f t="shared" si="1"/>
+        <v>79 - Ajuste en Pagos distintos a los listados y que no deben considerarse como ingreso por sueldos, salarios o ingresos asimilados.</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="33">
         <v>80</v>
       </c>
@@ -3765,8 +4419,12 @@
       </c>
       <c r="D85" s="14"/>
       <c r="E85" s="19"/>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85" t="str">
+        <f t="shared" si="1"/>
+        <v>80 - Ajuste en Viáticos gravados</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="33">
         <v>81</v>
       </c>
@@ -3778,8 +4436,12 @@
       </c>
       <c r="D86" s="14"/>
       <c r="E86" s="19"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86" t="str">
+        <f t="shared" si="1"/>
+        <v>81 - Ajuste en Viáticos (entregados al trabajador)</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="36" t="s">
         <v>167</v>
       </c>
@@ -3791,8 +4453,12 @@
       </c>
       <c r="D87" s="14"/>
       <c r="E87" s="19"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F87" t="str">
+        <f t="shared" si="1"/>
+        <v>82 - Ajuste en Fondo de ahorro Gravado</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="36" t="s">
         <v>169</v>
       </c>
@@ -3804,8 +4470,12 @@
       </c>
       <c r="D88" s="14"/>
       <c r="E88" s="19"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F88" t="str">
+        <f t="shared" si="1"/>
+        <v>83 - Ajuste en Caja de ahorro Gravado</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="36" t="s">
         <v>171</v>
       </c>
@@ -3817,8 +4487,12 @@
       </c>
       <c r="D89" s="14"/>
       <c r="E89" s="19"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F89" t="str">
+        <f t="shared" si="1"/>
+        <v>84 - Ajuste en Prima de Seguro de vida Gravado</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="36" t="s">
         <v>173</v>
       </c>
@@ -3830,8 +4504,12 @@
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="19"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F90" t="str">
+        <f t="shared" si="1"/>
+        <v>85 - Ajuste en Seguro de Gastos Médicos Mayores Gravado</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="36" t="s">
         <v>175</v>
       </c>
@@ -3843,8 +4521,12 @@
       </c>
       <c r="D91" s="14"/>
       <c r="E91" s="19"/>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F91" t="str">
+        <f t="shared" si="1"/>
+        <v>86 - Ajuste en Subsidios por incapacidad Gravado</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="36" t="s">
         <v>177</v>
       </c>
@@ -3856,8 +4538,12 @@
       </c>
       <c r="D92" s="14"/>
       <c r="E92" s="19"/>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F92" t="str">
+        <f t="shared" si="1"/>
+        <v>87 - Ajuste en Becas para trabajadores y/o hijos Gravado</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="36" t="s">
         <v>179</v>
       </c>
@@ -3869,8 +4555,12 @@
       </c>
       <c r="D93" s="14"/>
       <c r="E93" s="19"/>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F93" t="str">
+        <f t="shared" si="1"/>
+        <v>88 - Ajuste en Seguro de retiro Gravado</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="36" t="s">
         <v>181</v>
       </c>
@@ -3882,8 +4572,12 @@
       </c>
       <c r="D94" s="14"/>
       <c r="E94" s="19"/>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F94" t="str">
+        <f t="shared" si="1"/>
+        <v>89 - Ajuste en Vales de despensa Gravado</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="36" t="s">
         <v>183</v>
       </c>
@@ -3895,8 +4589,12 @@
       </c>
       <c r="D95" s="14"/>
       <c r="E95" s="19"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F95" t="str">
+        <f t="shared" si="1"/>
+        <v>90 - Ajuste en Vales de restaurante Gravado</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="36" t="s">
         <v>185</v>
       </c>
@@ -3908,8 +4606,12 @@
       </c>
       <c r="D96" s="14"/>
       <c r="E96" s="19"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F96" t="str">
+        <f t="shared" si="1"/>
+        <v>91 - Ajuste en Vales de gasolina Gravado</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="36" t="s">
         <v>187</v>
       </c>
@@ -3921,8 +4623,12 @@
       </c>
       <c r="D97" s="14"/>
       <c r="E97" s="19"/>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F97" t="str">
+        <f t="shared" si="1"/>
+        <v>92 - Ajuste en Vales de ropa Gravado</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="36" t="s">
         <v>189</v>
       </c>
@@ -3934,8 +4640,12 @@
       </c>
       <c r="D98" s="14"/>
       <c r="E98" s="19"/>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F98" t="str">
+        <f t="shared" si="1"/>
+        <v>93 - Ajuste en Ayuda para renta Gravado</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="36" t="s">
         <v>191</v>
       </c>
@@ -3947,8 +4657,12 @@
       </c>
       <c r="D99" s="14"/>
       <c r="E99" s="19"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F99" t="str">
+        <f t="shared" si="1"/>
+        <v>94 - Ajuste en Ayuda para artículos escolares Gravado</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="36" t="s">
         <v>193</v>
       </c>
@@ -3960,8 +4674,12 @@
       </c>
       <c r="D100" s="14"/>
       <c r="E100" s="19"/>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F100" t="str">
+        <f t="shared" si="1"/>
+        <v>95 - Ajuste en Ayuda para anteojos Gravado</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="36" t="s">
         <v>195</v>
       </c>
@@ -3973,8 +4691,12 @@
       </c>
       <c r="D101" s="14"/>
       <c r="E101" s="19"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F101" t="str">
+        <f t="shared" si="1"/>
+        <v>96 - Ajuste en Ayuda para transporte Gravado</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="36" t="s">
         <v>197</v>
       </c>
@@ -3986,8 +4708,12 @@
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="19"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F102" t="str">
+        <f t="shared" si="1"/>
+        <v>97 - Ajuste en Ayuda para gastos de funeral Gravado</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="36" t="s">
         <v>199</v>
       </c>
@@ -3999,8 +4725,12 @@
       </c>
       <c r="D103" s="14"/>
       <c r="E103" s="19"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F103" t="str">
+        <f t="shared" si="1"/>
+        <v>98 - Ajuste a ingresos asimilados a salarios gravados</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="36" t="s">
         <v>201</v>
       </c>
@@ -4012,8 +4742,12 @@
       </c>
       <c r="D104" s="14"/>
       <c r="E104" s="19"/>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F104" t="str">
+        <f t="shared" si="1"/>
+        <v>99 - Ajuste a ingresos por sueldos y salarios gravados</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="36">
         <v>100</v>
       </c>
@@ -4025,8 +4759,12 @@
       </c>
       <c r="D105" s="14"/>
       <c r="E105" s="19"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" t="str">
+        <f t="shared" si="1"/>
+        <v>100 - Ajuste en Viáticos exentos</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="36">
         <v>101</v>
       </c>
@@ -4038,8 +4776,12 @@
       </c>
       <c r="D106" s="14"/>
       <c r="E106" s="19"/>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F106" t="str">
+        <f t="shared" si="1"/>
+        <v>101 - ISR Retenido de ejercicio anterior</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="26">
         <v>102</v>
       </c>
@@ -4051,8 +4793,12 @@
       </c>
       <c r="D107" s="37"/>
       <c r="E107" s="19"/>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F107" t="str">
+        <f t="shared" si="1"/>
+        <v>102 - Ajuste a pagos por gratificaciones, primas, compensaciones, recompensas u otros a extrabajadores derivados de jubilación en parcialidades, gravados</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="26">
         <v>103</v>
       </c>
@@ -4064,8 +4810,12 @@
       </c>
       <c r="D108" s="37"/>
       <c r="E108" s="19"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F108" t="str">
+        <f t="shared" si="1"/>
+        <v>103 - Ajuste a pagos que se realicen a extrabajadores que obtengan una jubilación en parcialidades derivados de la ejecución de una resolución judicial o de un laudo gravados</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="26">
         <v>104</v>
       </c>
@@ -4077,8 +4827,12 @@
       </c>
       <c r="D109" s="37"/>
       <c r="E109" s="19"/>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F109" t="str">
+        <f t="shared" si="1"/>
+        <v>104 - Ajuste a pagos que se realicen a extrabajadores que obtengan una jubilación en parcialidades derivados de la ejecución de una resolución judicial o de un laudo exentos</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="26">
         <v>105</v>
       </c>
@@ -4090,8 +4844,12 @@
       </c>
       <c r="D110" s="37"/>
       <c r="E110" s="19"/>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F110" t="str">
+        <f t="shared" si="1"/>
+        <v>105 - Ajuste a pagos que se realicen a extrabajadores que obtengan una jubilación en una sola exhibición derivados de la ejecución de una resolución judicial o de un laudo gravados</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="26">
         <v>106</v>
       </c>
@@ -4103,8 +4861,12 @@
       </c>
       <c r="D111" s="37"/>
       <c r="E111" s="19"/>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F111" t="str">
+        <f t="shared" si="1"/>
+        <v>106 - Ajuste a pagos que se realicen a extrabajadores que obtengan una jubilación en una sola exhibición derivados de la ejecución de una resolución judicial o de un laudo exentos</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="26">
         <v>107</v>
       </c>
@@ -4116,6 +4878,10 @@
       </c>
       <c r="D112" s="37"/>
       <c r="E112" s="19"/>
+      <c r="F112" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">107 - Ajuste al Subsidio Causado </v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4128,7 +4894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5948F83A-D83D-4CC3-9C46-1FB670DFE456}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -4137,15 +4903,15 @@
     <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="87" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="72"/>
+      <c r="B1" s="87"/>
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>35</v>
       </c>
@@ -4157,7 +4923,7 @@
       </c>
       <c r="D2" s="19"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="28">
         <v>4</v>
       </c>
@@ -4169,13 +4935,13 @@
       </c>
       <c r="D3" s="19"/>
     </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19"/>
       <c r="B4" s="19"/>
       <c r="C4" s="19"/>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39" t="s">
         <v>212</v>
       </c>
@@ -4189,7 +4955,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <v>1</v>
       </c>
@@ -4200,8 +4966,12 @@
         <v>42736</v>
       </c>
       <c r="D6" s="38"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" t="str">
+        <f>VALUE(A6) &amp; " - " &amp; B6</f>
+        <v>1 - Reintegro de ISR pagado en exceso (siempre que no haya sido enterado al SAT).</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <v>2</v>
       </c>
@@ -4212,8 +4982,12 @@
         <v>42736</v>
       </c>
       <c r="D7" s="38"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" t="str">
+        <f t="shared" ref="F7:F15" si="0">VALUE(A7) &amp; " - " &amp; B7</f>
+        <v>2 - Subsidio para el empleo (efectivamente entregado al trabajador).</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <v>3</v>
       </c>
@@ -4224,8 +4998,12 @@
         <v>42736</v>
       </c>
       <c r="D8" s="38"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>3 - Viáticos (entregados al trabajador).</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <v>4</v>
       </c>
@@ -4236,8 +5014,12 @@
         <v>42736</v>
       </c>
       <c r="D9" s="38"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>4 - Aplicación de saldo a favor por compensación anual.</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <v>5</v>
       </c>
@@ -4248,8 +5030,12 @@
         <v>43074</v>
       </c>
       <c r="D10" s="38"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>5 - Reintegro de ISR retenido en exceso de ejercicio anterior (siempre que no haya sido enterado al SAT).</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <v>6</v>
       </c>
@@ -4260,8 +5046,12 @@
         <v>43831</v>
       </c>
       <c r="D11" s="38"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>6 - Alimentos en bienes (Servicios de comedor y comida) Art 94 último párrafo LISR.</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <v>7</v>
       </c>
@@ -4272,8 +5062,12 @@
         <v>43831</v>
       </c>
       <c r="D12" s="38"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>7 - ISR ajustado por subsidio.</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <v>8</v>
       </c>
@@ -4284,8 +5078,12 @@
         <v>43831</v>
       </c>
       <c r="D13" s="38"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>8 - Subsidio efectivamente entregado que no correspondía (Aplica sólo cuando haya ajuste al cierre de mes en relación con el Apéndice 7 de la guía de llenado de nómina).</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <v>9</v>
       </c>
@@ -4296,8 +5094,12 @@
         <v>43941</v>
       </c>
       <c r="D14" s="38"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>9 - Reembolso de descuentos efectuados para el crédito de vivienda.</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <v>999</v>
       </c>
@@ -4308,6 +5110,10 @@
         <v>42736</v>
       </c>
       <c r="D15" s="38"/>
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>999 - Pagos distintos a los listados y que no deben considerarse como ingreso por sueldos, salarios o ingresos asimilados.</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4319,7 +5125,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AABB6C07-4C11-4E3B-A6A8-42776ECFCA33}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
@@ -4328,15 +5134,15 @@
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="69" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="84" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
       <c r="D1" s="19"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>40</v>
       </c>
@@ -4350,7 +5156,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="29">
         <v>43831</v>
       </c>
@@ -4362,13 +5168,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19"/>
       <c r="B4" s="19"/>
       <c r="C4" s="19"/>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
         <v>224</v>
       </c>
@@ -4378,45 +5184,61 @@
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" t="str">
+        <f>VALUE(A6) &amp; " - "  &amp; B6</f>
+        <v>1 - Riesgo de trabajo</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C7" s="19"/>
       <c r="D7" s="19"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" t="str">
+        <f t="shared" ref="F7:F9" si="0">VALUE(A7) &amp; " - "  &amp; B7</f>
+        <v>2 - Enfermedad en general</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>3 - Maternidad</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="40" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="19"/>
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>4 - Licencia por cuidados médicos de hijos diagnosticados con cáncer</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
ajuste y modificaciones en la vista previa de nomina
</commit_message>
<xml_diff>
--- a/RN_GC/web/resources/Archivos/Plantilla_Nomina.xlsx
+++ b/RN_GC/web/resources/Archivos/Plantilla_Nomina.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaquin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Contador\Pruebas\Plantilla Ejemplo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6CB7C5-FCAC-4DA9-AF1C-2A167C87038A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E7DA36-5BEC-4756-B672-4C5A8ABDCBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6ABFC6CB-095B-4185-B39D-046E00DEABE2}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7785" xr2:uid="{6ABFC6CB-095B-4185-B39D-046E00DEABE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Timbrado" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="261">
   <si>
     <t>RFC PATRONAL:</t>
   </si>
@@ -732,6 +732,9 @@
     <t>04</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>No. Empleado</t>
   </si>
   <si>
@@ -745,6 +748,93 @@
   </si>
   <si>
     <t>Licencia por cuidados médicos de hijos diagnosticados con cáncer</t>
+  </si>
+  <si>
+    <t>Ingresos federales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMAR </t>
+  </si>
+  <si>
+    <t>MELENDEZ</t>
+  </si>
+  <si>
+    <t>POLVO</t>
+  </si>
+  <si>
+    <t>Sueldo</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Quincenal</t>
+  </si>
+  <si>
+    <t>1 - Sueldos, Salarios  Rayas y Jornales</t>
+  </si>
+  <si>
+    <t>2 - ISR</t>
+  </si>
+  <si>
+    <t>Nómina Ordinaria</t>
+  </si>
+  <si>
+    <t>3 - Aportaciones a retiro, cesantía en edad avanzada y vejez.</t>
+  </si>
+  <si>
+    <t>1 - Seguridad social</t>
+  </si>
+  <si>
+    <t>2 - Subsidio para el empleo (efectivamente entregado al trabajador).</t>
+  </si>
+  <si>
+    <t>ESCUELA DE ENFERMERIA FLORENCIA NIGHTINGALE TLAXCALA-TLAX</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>JUANA</t>
+  </si>
+  <si>
+    <t>MENESES</t>
+  </si>
+  <si>
+    <t>MORALES</t>
+  </si>
+  <si>
+    <t>ISR Sueldos y salarios</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Retencion RCV</t>
+  </si>
+  <si>
+    <t>Subsidio al empleo</t>
+  </si>
+  <si>
+    <t>46 - Ingresos asimilados a salarios</t>
+  </si>
+  <si>
+    <t>Retención ISR asimilados a salarios</t>
+  </si>
+  <si>
+    <t>F1318728103</t>
+  </si>
+  <si>
+    <t>01/01/2026</t>
+  </si>
+  <si>
+    <t>16/01/2026</t>
+  </si>
+  <si>
+    <t>15/01/2026</t>
+  </si>
+  <si>
+    <t>Nomina Ejemplo</t>
   </si>
 </sst>
 </file>
@@ -1154,9 +1244,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1511,7 +1599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41371BBB-4714-4DEA-AB6C-BE84DA670BD5}">
-  <dimension ref="A2:Y41"/>
+  <dimension ref="A2:Y40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
@@ -1543,7 +1631,9 @@
       </c>
       <c r="B2" s="78"/>
       <c r="C2" s="43"/>
-      <c r="D2" s="45"/>
+      <c r="D2" s="45" t="s">
+        <v>256</v>
+      </c>
       <c r="H2" s="81" t="s">
         <v>1</v>
       </c>
@@ -1556,7 +1646,9 @@
         <v>2</v>
       </c>
       <c r="B3" s="78"/>
-      <c r="D3" s="45"/>
+      <c r="D3" s="45" t="s">
+        <v>245</v>
+      </c>
       <c r="H3" s="54"/>
       <c r="I3" s="54"/>
       <c r="J3" s="54"/>
@@ -1571,7 +1663,10 @@
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="45"/>
+      <c r="D4" s="45" t="s">
+        <v>260</v>
+      </c>
+      <c r="E4" s="74"/>
       <c r="H4" s="53"/>
       <c r="I4" s="53"/>
       <c r="J4" s="53"/>
@@ -1585,14 +1680,18 @@
         <v>3</v>
       </c>
       <c r="B6" s="78"/>
-      <c r="D6" s="45"/>
+      <c r="D6" s="45" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="78" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="78"/>
-      <c r="D7" s="45"/>
+      <c r="D7" s="45" t="s">
+        <v>258</v>
+      </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1602,14 +1701,18 @@
         <v>5</v>
       </c>
       <c r="B8" s="52"/>
-      <c r="D8" s="45"/>
+      <c r="D8" s="45" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="78" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="78"/>
-      <c r="D9" s="45"/>
+      <c r="D9" s="45" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="78" t="s">
@@ -1617,7 +1720,9 @@
       </c>
       <c r="B10" s="78"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="46"/>
+      <c r="D10" s="46" t="s">
+        <v>237</v>
+      </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -1633,7 +1738,9 @@
       </c>
       <c r="B11" s="52"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="46"/>
+      <c r="D11" s="46" t="s">
+        <v>238</v>
+      </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -1648,7 +1755,9 @@
         <v>8</v>
       </c>
       <c r="B12" s="79"/>
-      <c r="D12" s="45"/>
+      <c r="D12" s="45" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="48"/>
@@ -1764,7 +1873,7 @@
       </c>
       <c r="T16" s="58"/>
       <c r="U16" s="55" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="V16" s="55" t="s">
         <v>25</v>
@@ -1778,25 +1887,59 @@
       <c r="Y16" s="64"/>
     </row>
     <row r="17" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="46"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
+      <c r="A17" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>234</v>
+      </c>
+      <c r="D17" s="46" t="s">
+        <v>235</v>
+      </c>
+      <c r="E17" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="46" t="s">
+        <v>239</v>
+      </c>
+      <c r="G17" s="46" t="s">
+        <v>236</v>
+      </c>
+      <c r="H17" s="59">
+        <v>3733.95</v>
+      </c>
+      <c r="I17" s="59">
+        <v>0</v>
+      </c>
       <c r="J17" s="68"/>
-      <c r="K17" s="74"/>
-      <c r="L17" s="49"/>
-      <c r="M17" s="46"/>
-      <c r="N17" s="59"/>
+      <c r="K17" s="73">
+        <v>2</v>
+      </c>
+      <c r="L17" s="49" t="s">
+        <v>240</v>
+      </c>
+      <c r="M17" s="46" t="s">
+        <v>250</v>
+      </c>
+      <c r="N17" s="59">
+        <v>249.77</v>
+      </c>
       <c r="O17" s="3"/>
-      <c r="P17" s="46"/>
-      <c r="Q17" s="46"/>
-      <c r="R17" s="46"/>
-      <c r="S17" s="59"/>
+      <c r="P17" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q17" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="R17" s="46" t="s">
+        <v>253</v>
+      </c>
+      <c r="S17" s="59">
+        <v>195.06</v>
+      </c>
       <c r="T17" s="57"/>
       <c r="U17" s="46"/>
       <c r="V17" s="46"/>
@@ -1804,20 +1947,46 @@
       <c r="X17" s="59"/>
     </row>
     <row r="18" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="46"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="59"/>
-      <c r="I18" s="59"/>
+      <c r="A18" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>247</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>248</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="46" t="s">
+        <v>254</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" s="59">
+        <v>2310</v>
+      </c>
+      <c r="I18" s="59">
+        <v>0</v>
+      </c>
       <c r="J18" s="68"/>
-      <c r="K18" s="73"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="46"/>
-      <c r="N18" s="59"/>
+      <c r="K18" s="71" t="s">
+        <v>226</v>
+      </c>
+      <c r="L18" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="M18" s="46" t="s">
+        <v>251</v>
+      </c>
+      <c r="N18" s="59">
+        <v>49.24</v>
+      </c>
       <c r="O18" s="3"/>
       <c r="P18" s="46"/>
       <c r="Q18" s="46"/>
@@ -1829,31 +1998,38 @@
       <c r="W18" s="46"/>
       <c r="X18" s="59"/>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="46"/>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A19" s="45"/>
       <c r="B19" s="46"/>
       <c r="C19" s="46"/>
       <c r="D19" s="46"/>
       <c r="E19" s="46"/>
       <c r="F19" s="46"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="59"/>
-      <c r="I19" s="59"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="60"/>
+      <c r="I19" s="60"/>
       <c r="J19" s="68"/>
-      <c r="K19" s="71"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="46"/>
-      <c r="N19" s="59"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="46"/>
+      <c r="K19" s="72" t="s">
+        <v>226</v>
+      </c>
+      <c r="L19" s="49" t="s">
+        <v>242</v>
+      </c>
+      <c r="M19" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="N19" s="60">
+        <v>44.31</v>
+      </c>
+      <c r="P19" s="45"/>
       <c r="Q19" s="46"/>
-      <c r="R19" s="46"/>
-      <c r="S19" s="59"/>
+      <c r="R19" s="45"/>
+      <c r="S19" s="60"/>
       <c r="T19" s="57"/>
       <c r="U19" s="46"/>
-      <c r="V19" s="46"/>
+      <c r="V19" s="45"/>
       <c r="W19" s="46"/>
-      <c r="X19" s="59"/>
+      <c r="X19" s="60"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" s="45"/>
@@ -1866,10 +2042,18 @@
       <c r="H20" s="60"/>
       <c r="I20" s="60"/>
       <c r="J20" s="68"/>
-      <c r="K20" s="72"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="45"/>
-      <c r="N20" s="60"/>
+      <c r="K20" s="72" t="s">
+        <v>246</v>
+      </c>
+      <c r="L20" s="49" t="s">
+        <v>240</v>
+      </c>
+      <c r="M20" s="46" t="s">
+        <v>255</v>
+      </c>
+      <c r="N20" s="60">
+        <v>114.41</v>
+      </c>
       <c r="P20" s="45"/>
       <c r="Q20" s="46"/>
       <c r="R20" s="45"/>
@@ -1909,7 +2093,7 @@
       <c r="A22" s="45"/>
       <c r="B22" s="46"/>
       <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
+      <c r="D22" s="63"/>
       <c r="E22" s="46"/>
       <c r="F22" s="46"/>
       <c r="G22" s="50"/>
@@ -1918,7 +2102,7 @@
       <c r="J22" s="68"/>
       <c r="K22" s="72"/>
       <c r="L22" s="49"/>
-      <c r="M22" s="46"/>
+      <c r="M22" s="50"/>
       <c r="N22" s="60"/>
       <c r="P22" s="45"/>
       <c r="Q22" s="46"/>
@@ -1931,20 +2115,17 @@
       <c r="X22" s="60"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A23" s="45"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="68"/>
-      <c r="K23" s="72"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="61"/>
       <c r="L23" s="49"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="60"/>
+      <c r="N23" s="61"/>
       <c r="P23" s="45"/>
       <c r="Q23" s="46"/>
       <c r="R23" s="45"/>
@@ -1959,61 +2140,49 @@
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="61"/>
-      <c r="I24" s="61"/>
-      <c r="J24" s="61"/>
-      <c r="K24" s="61"/>
-      <c r="L24" s="49"/>
-      <c r="N24" s="61"/>
-      <c r="P24" s="45"/>
-      <c r="Q24" s="46"/>
-      <c r="R24" s="45"/>
-      <c r="S24" s="60"/>
-      <c r="T24" s="57"/>
-      <c r="U24" s="46"/>
-      <c r="V24" s="45"/>
-      <c r="W24" s="46"/>
-      <c r="X24" s="60"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
       <c r="Q25" s="3"/>
       <c r="R25" s="3"/>
       <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
-      <c r="S26" s="3"/>
-      <c r="T26" s="3"/>
-      <c r="V26" s="3"/>
-      <c r="W26" s="3"/>
-      <c r="X26" s="3"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
+      <c r="J26" s="61"/>
+      <c r="K26" s="61"/>
+      <c r="N26" s="61"/>
+      <c r="S26" s="61"/>
+      <c r="V26" s="61"/>
+      <c r="X26" s="61"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="H27" s="61"/>
@@ -2041,7 +2210,7 @@
       <c r="J29" s="61"/>
       <c r="K29" s="61"/>
       <c r="N29" s="61"/>
-      <c r="S29" s="61"/>
+      <c r="S29" s="62"/>
       <c r="V29" s="61"/>
       <c r="X29" s="61"/>
     </row>
@@ -2051,7 +2220,7 @@
       <c r="J30" s="61"/>
       <c r="K30" s="61"/>
       <c r="N30" s="61"/>
-      <c r="S30" s="62"/>
+      <c r="S30" s="61"/>
       <c r="V30" s="61"/>
       <c r="X30" s="61"/>
     </row>
@@ -2081,8 +2250,6 @@
       <c r="J33" s="61"/>
       <c r="K33" s="61"/>
       <c r="N33" s="61"/>
-      <c r="S33" s="61"/>
-      <c r="V33" s="61"/>
       <c r="X33" s="61"/>
     </row>
     <row r="34" spans="8:24" x14ac:dyDescent="0.25">
@@ -2098,7 +2265,6 @@
       <c r="I35" s="61"/>
       <c r="J35" s="61"/>
       <c r="K35" s="61"/>
-      <c r="N35" s="61"/>
       <c r="X35" s="61"/>
     </row>
     <row r="36" spans="8:24" x14ac:dyDescent="0.25">
@@ -2113,7 +2279,6 @@
       <c r="I37" s="61"/>
       <c r="J37" s="61"/>
       <c r="K37" s="61"/>
-      <c r="X37" s="61"/>
     </row>
     <row r="38" spans="8:24" x14ac:dyDescent="0.25">
       <c r="H38" s="61"/>
@@ -2132,12 +2297,6 @@
       <c r="I40" s="61"/>
       <c r="J40" s="61"/>
       <c r="K40" s="61"/>
-    </row>
-    <row r="41" spans="8:24" x14ac:dyDescent="0.25">
-      <c r="H41" s="61"/>
-      <c r="I41" s="61"/>
-      <c r="J41" s="61"/>
-      <c r="K41" s="61"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -2189,31 +2348,31 @@
           <x14:formula1>
             <xm:f>TipoOtroPago!$F$6:$F$15</xm:f>
           </x14:formula1>
-          <xm:sqref>Q17:Q24</xm:sqref>
+          <xm:sqref>Q17:Q23</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E1BF81AA-AC21-476C-8F65-C86B9A11CE23}">
           <x14:formula1>
             <xm:f>Percepciones!$B$6:$B$49</xm:f>
           </x14:formula1>
-          <xm:sqref>E17:E23</xm:sqref>
+          <xm:sqref>E17:E22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56F2ED0B-3E68-4A97-A768-6C850C82DA62}">
           <x14:formula1>
             <xm:f>TipoIncapacidad!$F$6:$F$9</xm:f>
           </x14:formula1>
-          <xm:sqref>W17:W24</xm:sqref>
+          <xm:sqref>W17:W23</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{527D78B9-3CFD-41EB-B65D-D922748B021C}">
           <x14:formula1>
             <xm:f>Percepciones!$F$6:$F$49</xm:f>
           </x14:formula1>
-          <xm:sqref>F17:F23</xm:sqref>
+          <xm:sqref>F17:F22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0F30A284-2059-462B-A411-B81C0FC0D032}">
           <x14:formula1>
             <xm:f>Deducciones!$F$6:$F$112</xm:f>
           </x14:formula1>
-          <xm:sqref>L17:L24</xm:sqref>
+          <xm:sqref>L17:L23</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5189,7 +5348,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
@@ -5203,7 +5362,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C7" s="19"/>
       <c r="D7" s="19"/>
@@ -5217,7 +5376,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -5231,7 +5390,7 @@
         <v>225</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="19"/>

</xml_diff>